<commit_message>
Unify PP-PI into one Migration Blueprint Portal: web home IS the live cockpit (status->KPI/charts), each object row expands to its full technical blueprint (ops layer + fields + JOIN ON + guide); Excel relabeled, cockpit<->blueprint coupled via links
</commit_message>
<xml_diff>
--- a/SAP_PPPI_ECC6_to_S4_Migration.xlsx
+++ b/SAP_PPPI_ECC6_to_S4_Migration.xlsx
@@ -1266,7 +1266,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>CBC ISRAEL  |  SAP PP-PI  -  מסך ניווט מרכזי</t>
+          <t>CBC ISRAEL  |  SAP PP-PI Migration Blueprint Portal</t>
         </is>
       </c>
       <c r="C2" s="4" t="n"/>
@@ -1324,7 +1324,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Project NEO  -  Production Planning for Process Industries  |  ECC 6.0 ➜ S/4HANA</t>
+          <t>Project NEO  -  Migration Cockpit + Blueprint מאוחדים  |  PP-PI  ECC 6.0 ➜ S/4HANA</t>
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
@@ -1422,7 +1422,7 @@
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>סיכום התקדמות מיגרציה (KPI - חי מה-Cockpit)</t>
+          <t>🚀 Migration Cockpit - מצב פריסה חי (KPI מתעדכן מ-Cockpit; עדכן סטטוס בלשונית Cockpit, פתח Blueprint בלשוניות הזרמים)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>

</xml_diff>